<commit_message>
feat: adicionar semana 28 a 01, fechar setembro, iniciar outubro e recuperar 4803 pedidos em varredura backfill
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-16).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-16).xlsx
@@ -935,10 +935,10 @@
     <t>214</t>
   </si>
   <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>R$ 3.926,17</t>
+    <t>26</t>
+  </si>
+  <si>
+    <t>R$ 3.929,29</t>
   </si>
   <si>
     <t>43.7</t>
@@ -950,16 +950,16 @@
     <t>4.88</t>
   </si>
   <si>
-    <t>18.8</t>
-  </si>
-  <si>
-    <t>7.4</t>
+    <t>18.9</t>
+  </si>
+  <si>
+    <t>7.5</t>
   </si>
   <si>
     <t>6.2</t>
   </si>
   <si>
-    <t>41.6%</t>
+    <t>41.7%</t>
   </si>
   <si>
     <t>18.6%</t>
@@ -4961,7 +4961,7 @@
         <v>19536</v>
       </c>
       <c r="B24" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C24" s="4">
         <v>51</v>
@@ -4991,14 +4991,26 @@
         <v>58</v>
       </c>
       <c r="L24" s="4"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="6"/>
+      <c r="M24" s="5">
+        <v>4476.5200000000004</v>
+      </c>
+      <c r="N24" s="6">
+        <v>50</v>
+      </c>
       <c r="O24" s="6"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="8"/>
+      <c r="P24" s="7">
+        <v>4.831973469387755</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>25.160647222222224</v>
+      </c>
+      <c r="R24" s="8">
+        <v>13.464352777777778</v>
+      </c>
       <c r="S24" s="8"/>
-      <c r="T24" s="9"/>
+      <c r="T24" s="9">
+        <v>0.1111111111111111</v>
+      </c>
       <c r="U24" s="9"/>
       <c r="V24" s="9"/>
       <c r="W24" s="9"/>
@@ -14776,7 +14788,7 @@
         <v>19693</v>
       </c>
       <c r="B89" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C89" s="4">
         <v>51</v>
@@ -14804,14 +14816,26 @@
         <v>58</v>
       </c>
       <c r="L89" s="4"/>
-      <c r="M89" s="5"/>
-      <c r="N89" s="6"/>
+      <c r="M89" s="5">
+        <v>3958.8099999999999</v>
+      </c>
+      <c r="N89" s="6">
+        <v>37</v>
+      </c>
       <c r="O89" s="6"/>
-      <c r="P89" s="7"/>
-      <c r="Q89" s="8"/>
-      <c r="R89" s="8"/>
+      <c r="P89" s="7">
+        <v>4.1708333333333334</v>
+      </c>
+      <c r="Q89" s="8">
+        <v>22.87291875</v>
+      </c>
+      <c r="R89" s="8">
+        <v>9.3354187500000005</v>
+      </c>
       <c r="S89" s="8"/>
-      <c r="T89" s="9"/>
+      <c r="T89" s="9">
+        <v>0.125</v>
+      </c>
       <c r="U89" s="9"/>
       <c r="V89" s="9"/>
       <c r="W89" s="9"/>

</xml_diff>